<commit_message>
Reopen multi-platform monitoring (Blocked->Partial) per tested map
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/export/BFT_Living_Database.xlsx
+++ b/export/BFT_Living_Database.xlsx
@@ -44432,12 +44432,12 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Ask: continuously scan Facebook, X, Instagram, LinkedIn, Reddit, Pinterest, Minds, GETTR, MeWe, Gab, Telegram, Truth Social, Threads, Parler, Bluesky, YouTube, Rumble, Odysee, BitChute, TikTok for emerging pro-Israel voices. Claude only acts inside a turn -- there is no background monitoring.</t>
+          <t>REOPENED 17 Jul 2026 -- was wrongly marked Blocked on an untested assumption. TESTED: YouTube, Rumble, Gab, Threads, Bluesky (API), Telegram, and TikTok all fetch WITHOUT login; X works via the browser; Instagram/LinkedIn/Facebook need a login (now a solved assist workflow); the JS-rendered ones (Truth Social/GETTR/Twitch/etc) remain to browser-confirm. Original note follows. Ask: continuously scan Facebook, X, Instagram, LinkedIn, Reddit, Pinterest, Minds, GETTR, MeWe, Gab, Telegram, Truth Social, Threads, Parler, Bluesky, YouTube, Rumble, Odysee, BitChute, TikTok for emerging pro-Israel voices. Claude only acts inside a turn -- there is no background monitoring.</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Log decision: no stealth/anti-detect scraping of IG/LinkedIn (ToS); legitimate paths noted
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/export/BFT_Living_Database.xlsx
+++ b/export/BFT_Living_Database.xlsx
@@ -27,7 +27,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'political'!$A$1:$O$131</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'sponsor'!$A$1:$G$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'israeli_tech'!$A$1:$L$39</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'backlog'!$A$1:$G$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'backlog'!$A$1:$G$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'nurture'!$A$1:$R$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'criteria'!$A$1:$F$94</definedName>
   </definedNames>
@@ -823,7 +823,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>65 records</t>
+          <t>66 records</t>
         </is>
       </c>
     </row>
@@ -44416,7 +44416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G66"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -46822,8 +46822,41 @@
         </is>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr"/>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>DECISION: no stealth/anti-detect scraping of Instagram/LinkedIn</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="inlineStr">
+        <is>
+          <t>Blocked (Access/Ethics)</t>
+        </is>
+      </c>
+      <c r="D67" s="6" t="inlineStr">
+        <is>
+          <t>Needs Andy</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="inlineStr">
+        <is>
+          <t>Andy, 17 Jul 2026, asked whether a stealth/anti-detect browser tool (he named 'openclaw' -- not a tool Claude recognizes) could make Instagram/LinkedIn 'think it's me browsing not a bot.' TWO honest points. (1) The actual blocks were NOT bot-detection: the Claude-in-Chrome tool refuses to navigate to any domain in this env, and the in-app browser hits IG's logged-out login wall -- an anti-detect tool addresses neither. (2) Tools that exist for this (Playwright+stealth, undetected-chromedriver, anti-detect browsers, Apify/Bright Data) COULD read IG/LinkedIn with Andy's session, but their purpose is to DEFEAT the platform's bot detection, which violates Instagram/LinkedIn ToS (LinkedIn especially -- cf. hiQ v. LinkedIn). Claude will not engineer detection-evasion tooling; the goal (public figures' public counts) is legitimate, the evasion method is not.</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="inlineStr">
+        <is>
+          <t>LEGITIMATE PATHS to the same data, recommended in order: (1) the 6 platforms that already work logged-out (X/Gab/Threads/Bluesky/Telegram/YouTube/Rumble) cover most of the roster; (2) Andy pastes the ~10 highest-value Instagram/LinkedIn numbers he can see in his own browser -- zero ToS issue, works today; (3) official APIs (Instagram Graph API, LinkedIn API) for sanctioned scale access; (4) licensed providers (Social Blade / Apify official datasets) that handle ToS. RECOMMENDATION: do NOT build a stealth scraper for two holdout platforms -- the ToS/legal exposure is not worth it for an org that 'operates under the radar.' Revisit via official APIs only if IG/LinkedIn become a scale need.</t>
+        </is>
+      </c>
+      <c r="G67" s="6" t="inlineStr">
+        <is>
+          <t>Andy, 17 Jul 2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G66"/>
+  <autoFilter ref="A1:G67"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>